<commit_message>
luna56: rerun the 12 cases on the updated tests and update summaries
gpt-5.6-luna passes all 12 updated tests: 40/73 cases pass on every version, 43 on at least one, 546/1015 pairs (53.8%). Updated results CSV, wide summary CSV, xlsx (Relaxed Tests sheet removed), SUMMARY_luna56.md, logs, and run_output_luna56_updated_tests.txt.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Part3_LLM_repair/results/luna56/llm_luna56_summary.xlsx
+++ b/Part3_LLM_repair/results/luna56/llm_luna56_summary.xlsx
@@ -9,7 +9,6 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Stats &amp; Notes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Test Review" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Relaxed Tests" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -5292,119 +5291,119 @@
           <t>NOT_TESTED</t>
         </is>
       </c>
-      <c r="F15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="H15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="I15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="J15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="L15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="M15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="N15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="O15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="P15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="Q15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="R15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="S15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="T15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="U15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="V15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="W15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="X15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="Y15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="Z15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AA15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AB15" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="F15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="S15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="V15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="X15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Y15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Z15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AA15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AB15" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AC15" s="55" t="n"/>
@@ -12393,64 +12392,64 @@
           <t>issue_622</t>
         </is>
       </c>
-      <c r="B38" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="C38" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="D38" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="E38" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="F38" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G38" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="H38" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="I38" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="J38" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K38" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="L38" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="M38" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="B38" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C38" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D38" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E38" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F38" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G38" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H38" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I38" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J38" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K38" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L38" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M38" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="N38" s="56" t="inlineStr">
@@ -14120,139 +14119,139 @@
           <t>issue_671</t>
         </is>
       </c>
-      <c r="B43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="C43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="D43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="E43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="F43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="H43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="I43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="J43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="L43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="M43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="N43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="O43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="P43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="Q43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="R43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="S43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="T43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="U43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="V43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="W43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="X43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="Y43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="Z43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AA43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AB43" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="B43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="S43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="V43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="X43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Y43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Z43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AA43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AB43" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AC43" s="55" t="inlineStr">
@@ -15133,44 +15132,44 @@
           <t>NOT_TESTED</t>
         </is>
       </c>
-      <c r="F46" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G46" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="H46" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="I46" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="J46" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K46" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="L46" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="M46" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="F46" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G46" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H46" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I46" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J46" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K46" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L46" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M46" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="N46" s="56" t="inlineStr">
@@ -16557,64 +16556,64 @@
           <t>issue_775</t>
         </is>
       </c>
-      <c r="B50" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="C50" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D50" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="E50" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="F50" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="G50" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="H50" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="I50" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="J50" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="K50" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="L50" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="M50" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="B50" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C50" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D50" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E50" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F50" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G50" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H50" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I50" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J50" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K50" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L50" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M50" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="N50" s="56" t="inlineStr">
@@ -17539,9 +17538,9 @@
           <t>NOT_TESTED</t>
         </is>
       </c>
-      <c r="G53" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="G53" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H53" s="56" t="inlineStr">
@@ -17564,9 +17563,9 @@
           <t>NOT_TESTED</t>
         </is>
       </c>
-      <c r="L53" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="L53" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M53" s="56" t="inlineStr">
@@ -18726,14 +18725,14 @@
           <t>NOT_TESTED</t>
         </is>
       </c>
-      <c r="F57" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G57" s="58" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="F57" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G57" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H57" s="56" t="inlineStr">
@@ -19340,119 +19339,119 @@
           <t>NOT_TESTED</t>
         </is>
       </c>
-      <c r="F59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="G59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="H59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="I59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="J59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="K59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="L59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="M59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="N59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="O59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="P59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="Q59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="R59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="S59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="T59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="U59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="V59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="W59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="X59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="Y59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="Z59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="AA59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="AB59" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="F59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="S59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="V59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="X59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Y59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Z59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AA59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AB59" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AC59" s="55" t="n"/>
@@ -20090,64 +20089,64 @@
           <t>issue_944</t>
         </is>
       </c>
-      <c r="B61" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="C61" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D61" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="E61" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="F61" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="G61" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="H61" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="I61" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="J61" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="K61" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="L61" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="M61" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="B61" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C61" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D61" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E61" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F61" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G61" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H61" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I61" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J61" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K61" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L61" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M61" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="N61" s="56" t="inlineStr">
@@ -21523,119 +21522,119 @@
           <t>NOT_TESTED</t>
         </is>
       </c>
-      <c r="F64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="G64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="H64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="I64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="J64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="K64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="L64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="M64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="N64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="O64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="P64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="Q64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="R64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="S64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="T64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="U64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="V64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="W64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="X64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="Y64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="Z64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="AA64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="AB64" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="F64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="S64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="V64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="W64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="X64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Y64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Z64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AA64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AB64" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AC64" s="55" t="n"/>
@@ -22724,24 +22723,24 @@
           <t>issue_994</t>
         </is>
       </c>
-      <c r="B67" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="C67" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D67" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="E67" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="B67" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C67" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D67" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E67" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F67" s="56" t="inlineStr">
@@ -23015,44 +23014,44 @@
           <t>NOT_TESTED</t>
         </is>
       </c>
-      <c r="F68" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="G68" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="H68" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="I68" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="J68" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="K68" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="L68" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="M68" s="57" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="F68" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G68" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H68" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I68" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J68" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K68" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L68" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M68" s="59" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="N68" s="56" t="inlineStr">
@@ -25221,7 +25220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S264"/>
+  <dimension ref="A1:S263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="35" min="1" max="1"/>
@@ -25240,7 +25239,7 @@
     <row r="1">
       <c r="A1" s="60" t="inlineStr">
         <is>
-          <t>LLM bug-repair results (gpt-5.6-luna), judged by each case's test (test_new.py / test-new.py for issue_021_se, issue_058_se and issue_061; test.py for the rest)</t>
+          <t>LLM bug-repair results (gpt-5.6-luna), judged by each case's test (test_new.py / test-new.py for issue_021_se, issue_058_se and issue_061; test.py for the rest) Since 9 Oct 2026, the test.py of 12 over-specific cases holds an updated test that replaced the old one.</t>
         </is>
       </c>
     </row>
@@ -25251,6 +25250,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -25714,6 +25714,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="60" t="inlineStr">
         <is>
@@ -28766,6 +28767,7 @@
         <v>8</v>
       </c>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="60" t="inlineStr">
         <is>
@@ -29193,6 +29195,7 @@
         </is>
       </c>
     </row>
+    <row r="95"/>
     <row r="96">
       <c r="A96" s="60" t="inlineStr">
         <is>
@@ -31476,6 +31479,7 @@
         <v/>
       </c>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="60" t="inlineStr">
         <is>
@@ -32114,9 +32118,9 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="69" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="A198" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B198" s="67" t="inlineStr">
@@ -32132,19 +32136,11 @@
       <c r="D198" s="67" t="n">
         <v>23</v>
       </c>
-      <c r="E198" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError</t>
-        </is>
-      </c>
-      <c r="F198" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError: Lists differ: [2, 3, 4, 5, 6, 7, 8] != [0, 3, 4, 5, 6, 7, 8]</t>
-        </is>
-      </c>
+      <c r="E198" s="67" t="n"/>
+      <c r="F198" s="67" t="n"/>
       <c r="G198" s="67" t="inlineStr">
         <is>
-          <t>The LLM fixed the qubit count (one control plus the six target qubits) but kept the original code's control order, so control qubit k gets the power 2^k (the usual QPE layout, and every gate matrix is correct). The test only accepts the Stack Overflow answer's order (control i gets 2^(2-i)), so it reports [2, 3, ..., 8] instead of [0, 3, ..., 8].</t>
+          <t>Passed: the LLM fixed the qubit count (one control qubit plus the six target qubits) and kept the original control order, so control qubit k gets the power 2^k (the usual QPE layout). The updated test accepts either control order.</t>
         </is>
       </c>
       <c r="H198" s="67" t="n">
@@ -32908,9 +32904,9 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="69" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="A221" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B221" s="67" t="inlineStr">
@@ -32926,19 +32922,11 @@
       <c r="D221" s="67" t="n">
         <v>12</v>
       </c>
-      <c r="E221" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError</t>
-        </is>
-      </c>
-      <c r="F221" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError: Items in the first set but not the second: '01' '10'</t>
-        </is>
-      </c>
+      <c r="E221" s="67" t="n"/>
+      <c r="F221" s="67" t="n"/>
       <c r="G221" s="67" t="inlineStr">
         <is>
-          <t>The LLM swapped the 1-qubit FakeArmonk for the 5-qubit FakeYorktown, which fixes the qubit-count error, but fake backends simulate the device's noise, so about 9% of shots come out as '01' or '10'. The test requires only '00' and '11' (a noise-free simulator, like the reference's Aer qasm_simulator); every other check passes.</t>
+          <t>Passed: the LLM swapped the 1-qubit FakeArmonk for the 5-qubit FakeYorktown, so the Bell circuit runs on a large enough local backend. The updated test allows the fake device's noise.</t>
         </is>
       </c>
       <c r="H221" s="67" t="n">
@@ -33362,9 +33350,9 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="69" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="A234" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B234" s="67" t="inlineStr">
@@ -33380,19 +33368,11 @@
       <c r="D234" s="67" t="n">
         <v>27</v>
       </c>
-      <c r="E234" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError</t>
-        </is>
-      </c>
-      <c r="F234" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError: Not equal to tolerance rtol=1e-07, atol=1e-10</t>
-        </is>
-      </c>
+      <c r="E234" s="67" t="n"/>
+      <c r="F234" s="67" t="n"/>
       <c r="G234" s="67" t="inlineStr">
         <is>
-          <t>The LLM unpacked the list with QuantumCircuit(a, *v, b), which builds exactly the registers the question asks for, and every register check passes. The test then compares the full 512x512 unitary against the answer's example gates x(v0[0]) and cx(v1[0], a[0]), which are not in the buggy code. Without that unitary check the LLM fix passes (checked on 0.25.0, 0.45.3, 1.0.0, 1.2.4 and 2.5.0) and the buggy code still fails.</t>
+          <t>Passed: the LLM unpacked the list with QuantumCircuit(a, *v, b), which builds exactly the registers the question asks for (a, v0..v3, b in that order). The updated test checks the registers, not the answer's example gates.</t>
         </is>
       </c>
       <c r="H234" s="67" t="n">
@@ -33400,9 +33380,9 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="69" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="A235" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B235" s="67" t="inlineStr">
@@ -33418,19 +33398,11 @@
       <c r="D235" s="67" t="n">
         <v>8</v>
       </c>
-      <c r="E235" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError</t>
-        </is>
-      </c>
-      <c r="F235" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError: Items in the first set but not the second: '000 000' '111 000' Items in the second set but not the first: '000' '111'</t>
-        </is>
-      </c>
+      <c r="E235" s="67" t="n"/>
+      <c r="F235" s="67" t="n"/>
       <c r="G235" s="67" t="inlineStr">
         <is>
-          <t>The LLM added circ.measure_all(), which measures the GHZ state correctly but adds a second 3-bit register instead of using the circuit's existing 3 classical bits, so the counts keys are '000 000' / '111 000' instead of '000' / '111'. The reference measures into the existing bits. A test that ignores the unused register passes the LLM fix (checked on 0.45.0 and 0.46.3).</t>
+          <t>Passed: the LLM added circ.measure_all(), which measures the GHZ state correctly but adds a second register, so the count keys are '000 000' / '111 000'. The updated test accepts any register layout.</t>
         </is>
       </c>
       <c r="H235" s="67" t="n">
@@ -33514,9 +33486,9 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="70" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="A238" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B238" s="67" t="inlineStr">
@@ -33532,19 +33504,11 @@
       <c r="D238" s="67" t="n">
         <v>12</v>
       </c>
-      <c r="E238" s="67" t="inlineStr">
-        <is>
-          <t>KeyError</t>
-        </is>
-      </c>
-      <c r="F238" s="67" t="inlineStr">
-        <is>
-          <t>KeyError: 'qc'</t>
-        </is>
-      </c>
+      <c r="E238" s="67" t="n"/>
+      <c r="F238" s="67" t="n"/>
       <c r="G238" s="67" t="inlineStr">
         <is>
-          <t>The LLM parsed the QASM with QuantumCircuit.from_qasm_str and executed it, which is the right fix, but inlined the call inside execute(...) instead of storing it in a variable. The test reads the variable qc, so it raises KeyError. A test that checks the executed result instead passes the LLM fix (checked on 0.25.0, 0.45.0 and 0.46.3) and still fails the buggy code.</t>
+          <t>Passed: the LLM parsed the QASM with QuantumCircuit.from_qasm_str() and executed it. The updated test checks the executed result instead of a variable named qc.</t>
         </is>
       </c>
       <c r="H238" s="67" t="n">
@@ -33620,9 +33584,9 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="69" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="A241" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B241" s="67" t="inlineStr">
@@ -33638,19 +33602,11 @@
       <c r="D241" s="67" t="n">
         <v>2</v>
       </c>
-      <c r="E241" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError</t>
-        </is>
-      </c>
-      <c r="F241" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError: None is not an instance of &lt;class 'dict'&gt; : Expose a raw counts dictionary, not the Result object</t>
-        </is>
-      </c>
+      <c r="E241" s="67" t="n"/>
+      <c r="F241" s="67" t="n"/>
       <c r="G241" s="67" t="inlineStr">
         <is>
-          <t>The LLM replaced job.result(job) with job.result().get_counts(), the same call as the reference. The test reads the reference's variable name counts_dict and expects exactly 100 shots (the reference changed 1024 to 100), so it finds None. A test that accepts any variable name and the script's own shot count passes the LLM fix (checked on 0.45.1 and 0.46.2) and still fails the buggy code.</t>
+          <t>Passed: the LLM replaced job.result(job) with job.result().get_counts(), which returns the raw counts dictionary, the same call as the reference. The updated test accepts any variable name and the script's own shot count.</t>
         </is>
       </c>
       <c r="H241" s="67" t="n">
@@ -33658,9 +33614,9 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="69" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="A242" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B242" s="67" t="inlineStr">
@@ -33676,19 +33632,11 @@
       <c r="D242" s="67" t="n">
         <v>2</v>
       </c>
-      <c r="E242" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError</t>
-        </is>
-      </c>
-      <c r="F242" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError: {'00 00': 1024} != {'00': 1024}</t>
-        </is>
-      </c>
+      <c r="E242" s="67" t="n"/>
+      <c r="F242" s="67" t="n"/>
       <c r="G242" s="67" t="inlineStr">
         <is>
-          <t>The LLM transpiled the circuit before running it, which is the answer's fix. It kept the buggy code's QuantumCircuit(2, 2) plus measure_all(), so the keys are '00 00' instead of '00' (the reference also removed the classical register), and it did not store the transpiled circuit in transpile_circ. A test that ignores the unused register and the variable name passes the LLM fix (checked on 0.45.0 and 0.45.1).</t>
+          <t>Passed: the LLM transpiled the circuit before running it on qasm_simulator, the fix the answer gives. The updated test checks the job result regardless of the unused classical register and the variable name.</t>
         </is>
       </c>
       <c r="H242" s="67" t="n">
@@ -33886,9 +33834,9 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="70" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="A248" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B248" s="67" t="inlineStr">
@@ -33898,25 +33846,17 @@
       </c>
       <c r="C248" s="67" t="inlineStr">
         <is>
-          <t>0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3, 1.0.0, 1.0.1, 1.0.2, 1.1.0, 1.1.1, 1.1.2, 1.2.0, 1.2.1, 1.2.2, 1.2.4</t>
+          <t>0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3, 1.0.0, 1.0.1, 1.0.2, 1.1.0, 1.1.1, 1.1.2, 1.2.0, 1.2.1, 1.2.2, 1.2.4, 2.0.0, 2.2.0, 2.3.0, 2.4.0, 2.5.0</t>
         </is>
       </c>
       <c r="D248" s="67" t="n">
-        <v>18</v>
-      </c>
-      <c r="E248" s="67" t="inlineStr">
-        <is>
-          <t>ValueError</t>
-        </is>
-      </c>
-      <c r="F248" s="67" t="inlineStr">
-        <is>
-          <t>ValueError: malformed node or string on line 1: &lt;ast.Call object at 0x000001994F5AB2E0&gt;</t>
-        </is>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="E248" s="67" t="n"/>
+      <c r="F248" s="67" t="n"/>
       <c r="G248" s="67" t="inlineStr">
         <is>
-          <t>The LLM printed each qubit's register and index with qc.find_bit(), the information the question asks for. The test parses the reference's exact print format ('qargs : [0, 1]'), and the LLM's 'qargs :' line still prints Qubit objects, so ast.literal_eval raises ValueError. A test that reads the printed indices in either format passes the LLM fix (checked on 0.45.0, 1.0.0, 1.2.4 and 2.5.0).</t>
+          <t>Passed: the LLM looped over every operand and printed each qubit's register and index with qc.find_bit(). The updated test reads the printed indices in any format.</t>
         </is>
       </c>
       <c r="H248" s="67" t="n">
@@ -33931,30 +33871,30 @@
       </c>
       <c r="B249" s="67" t="inlineStr">
         <is>
-          <t>issue_911</t>
+          <t>issue_925</t>
         </is>
       </c>
       <c r="C249" s="67" t="inlineStr">
         <is>
-          <t>2.0.0, 2.2.0, 2.3.0, 2.4.0, 2.5.0</t>
+          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3</t>
         </is>
       </c>
       <c r="D249" s="67" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E249" s="67" t="inlineStr">
         <is>
-          <t>SyntaxError</t>
+          <t>TranspilerError</t>
         </is>
       </c>
       <c r="F249" s="67" t="inlineStr">
         <is>
-          <t>SyntaxError: invalid syntax</t>
+          <t>qiskit.transpiler.exceptions.TranspilerError: 'Number of qubits (18) in Shor(N=15, a=2) is greater than maximum (14) in the coupling_map'</t>
         </is>
       </c>
       <c r="G249" s="67" t="inlineStr">
         <is>
-          <t>Same fix and same test problem as on the older versions; in Qiskit 2.x the Qubit objects print in a form ast.literal_eval cannot read, so it raises SyntaxError instead.</t>
+          <t>The LLM only added a comment saying to use a simulator with enough qubits; the code still runs Shor on FakeMelbourne, so the 18-qubit circuit does not fit its 14-qubit coupling map, exactly like the buggy code. The reference switches to Aer's qasm_simulator.</t>
         </is>
       </c>
       <c r="H249" s="67" t="n">
@@ -33962,37 +33902,29 @@
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="70" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="A250" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B250" s="67" t="inlineStr">
         <is>
-          <t>issue_925</t>
+          <t>issue_944</t>
         </is>
       </c>
       <c r="C250" s="67" t="inlineStr">
         <is>
-          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3</t>
+          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3, 0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3</t>
         </is>
       </c>
       <c r="D250" s="67" t="n">
-        <v>4</v>
-      </c>
-      <c r="E250" s="67" t="inlineStr">
-        <is>
-          <t>TranspilerError</t>
-        </is>
-      </c>
-      <c r="F250" s="67" t="inlineStr">
-        <is>
-          <t>qiskit.transpiler.exceptions.TranspilerError: 'Number of qubits (18) in Shor(N=15, a=2) is greater than maximum (14) in the coupling_map'</t>
-        </is>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="E250" s="67" t="n"/>
+      <c r="F250" s="67" t="n"/>
       <c r="G250" s="67" t="inlineStr">
         <is>
-          <t>The LLM only added a comment saying to use a simulator with enough qubits; the code still runs Shor on FakeMelbourne, so the 18-qubit circuit does not fit its 14-qubit coupling map, exactly like the buggy code. The reference switches to Aer's qasm_simulator.</t>
+          <t>Passed: the LLM built |+&gt;&lt;+| as the opflow operator (I + X) / 2 and passed it to NumPyEigensolver, which gives the right projector and eigenvalues. The updated test accepts either operator type.</t>
         </is>
       </c>
       <c r="H250" s="67" t="n">
@@ -34000,67 +33932,67 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="70" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="A251" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B251" s="67" t="inlineStr">
         <is>
-          <t>issue_944</t>
+          <t>issue_989</t>
         </is>
       </c>
       <c r="C251" s="67" t="inlineStr">
         <is>
-          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3, 0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3</t>
+          <t>1.0.0, 1.0.1, 1.0.2, 1.1.0, 1.1.1, 1.1.2, 1.2.0, 1.2.1, 1.2.2, 1.2.4, 2.0.0, 2.2.0, 2.3.0, 2.4.0, 2.5.0</t>
         </is>
       </c>
       <c r="D251" s="67" t="n">
-        <v>12</v>
-      </c>
-      <c r="E251" s="67" t="inlineStr">
-        <is>
-          <t>AttributeError</t>
-        </is>
-      </c>
-      <c r="F251" s="67" t="inlineStr">
-        <is>
-          <t>AttributeError: 'PauliSumOp' object has no attribute 'data'</t>
-        </is>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="E251" s="67" t="n"/>
+      <c r="F251" s="67" t="n"/>
       <c r="G251" s="67" t="inlineStr">
         <is>
-          <t>The LLM built |+&gt;&lt;+| as the opflow operator (I + X) / 2 and passed it to NumPyEigensolver, which gives the right projector and eigenvalues. The test reads proj.data, which only the reference's quantum_info Operator has (and a variable named op). A test that accepts either operator type passes the LLM fix (checked on 0.25.0, 0.45.0 and 0.46.3) and still fails the buggy code.</t>
+          <t>The LLM changed the import to from qiskit_aer import Aer, the same fix as the reference.</t>
         </is>
       </c>
       <c r="H251" s="67" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="68" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="A252" s="69" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="B252" s="67" t="inlineStr">
         <is>
-          <t>issue_989</t>
+          <t>issue_950</t>
         </is>
       </c>
       <c r="C252" s="67" t="inlineStr">
         <is>
-          <t>1.0.0, 1.0.1, 1.0.2, 1.1.0, 1.1.1, 1.1.2, 1.2.0, 1.2.1, 1.2.2, 1.2.4, 2.0.0, 2.2.0, 2.3.0, 2.4.0, 2.5.0</t>
+          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3, 0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3, 1.0.0, 1.0.1, 1.0.2, 1.1.0, 1.1.1, 1.1.2, 1.2.0, 1.2.1, 1.2.2, 1.2.4, 2.0.0, 2.2.0, 2.3.0, 2.4.0, 2.5.0</t>
         </is>
       </c>
       <c r="D252" s="67" t="n">
-        <v>15</v>
-      </c>
-      <c r="E252" s="67" t="n"/>
-      <c r="F252" s="67" t="n"/>
+        <v>27</v>
+      </c>
+      <c r="E252" s="67" t="inlineStr">
+        <is>
+          <t>AssertionError</t>
+        </is>
+      </c>
+      <c r="F252" s="67" t="inlineStr">
+        <is>
+          <t>AssertionError: Not equal to tolerance rtol=1e-07, atol=1e-12 | AssertionError: Not equal to tolerance rtol=1e-07, atol=1e-12 Requested Z on qubits 3..7, not on qubits 2..6 Mismatched elements: 1024 / 1024 (100%) Max absolute difference: 1. Max relat</t>
+        </is>
+      </c>
       <c r="G252" s="67" t="inlineStr">
         <is>
-          <t>The LLM changed the import to from qiskit_aer import Aer, the same fix as the reference.</t>
+          <t>The LLM made the identity N qubits wide, which removes the size mismatch, but kept Operator._add(), which adds the operators instead of placing Z on qubits 3 to 7. The result is I + Z...Z, with 2 and 0 on the diagonal instead of +1 and -1. The reference builds the full Pauli label and calls Operator.from_label once.</t>
         </is>
       </c>
       <c r="H252" s="67" t="n">
@@ -34075,16 +34007,16 @@
       </c>
       <c r="B253" s="67" t="inlineStr">
         <is>
-          <t>issue_950</t>
+          <t>issue_958</t>
         </is>
       </c>
       <c r="C253" s="67" t="inlineStr">
         <is>
-          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3, 0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3, 1.0.0, 1.0.1, 1.0.2, 1.1.0, 1.1.1, 1.1.2, 1.2.0, 1.2.1, 1.2.2, 1.2.4, 2.0.0, 2.2.0, 2.3.0, 2.4.0, 2.5.0</t>
+          <t>0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3, 1.0.0, 1.0.1, 1.0.2, 1.1.0, 1.1.1, 1.1.2, 1.2.0, 1.2.1, 1.2.2, 1.2.4, 2.0.0, 2.2.0, 2.3.0, 2.4.0, 2.5.0</t>
         </is>
       </c>
       <c r="D253" s="67" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E253" s="67" t="inlineStr">
         <is>
@@ -34093,12 +34025,12 @@
       </c>
       <c r="F253" s="67" t="inlineStr">
         <is>
-          <t>AssertionError: Not equal to tolerance rtol=1e-07, atol=1e-12 | AssertionError: Not equal to tolerance rtol=1e-07, atol=1e-12 Requested Z on qubits 3..7, not on qubits 2..6 Mismatched elements: 1024 / 1024 (100%) Max absolute difference: 1. Max relat</t>
+          <t>AssertionError: Not equal to tolerance rtol=1e-07, atol=1e-12</t>
         </is>
       </c>
       <c r="G253" s="67" t="inlineStr">
         <is>
-          <t>The LLM made the identity N qubits wide, which removes the size mismatch, but kept Operator._add(), which adds the operators instead of placing Z on qubits 3 to 7. The result is I + Z...Z, with 2 and 0 on the diagonal instead of +1 and -1. The reference builds the full Pauli label and calls Operator.from_label once.</t>
+          <t>The LLM replaced -1 * gate1 with gate1([0, 1]).inverse(), which applies H to both qubits a second time. H twice is the identity, so the circuit is I instead of -(H x H) and the -1 phase never appears. The test also expects the reference's second circuit qc2, but the LLM fix already fails the check on qc. The reference adds a GlobalPhaseGate(pi).</t>
         </is>
       </c>
       <c r="H253" s="67" t="n">
@@ -34113,7 +34045,7 @@
       </c>
       <c r="B254" s="67" t="inlineStr">
         <is>
-          <t>issue_958</t>
+          <t>issue_985</t>
         </is>
       </c>
       <c r="C254" s="67" t="inlineStr">
@@ -34136,7 +34068,7 @@
       </c>
       <c r="G254" s="67" t="inlineStr">
         <is>
-          <t>The LLM replaced -1 * gate1 with gate1([0, 1]).inverse(), which applies H to both qubits a second time. H twice is the identity, so the circuit is I instead of -(H x H) and the -1 phase never appears. The test also expects the reference's second circuit qc2, but the LLM fix already fails the check on qc. The reference adds a GlobalPhaseGate(pi).</t>
+          <t>The LLM replaced u1 with rz and set qc.global_phase = lam / 2, so the transpiled circuit uses only rx/ry/rz and equals U1(0.5) exactly, phase included, as the question asks. The current test requires the phase to be missing (determinant 1), following the answer's point that rotations alone cannot carry it. The team's earlier test_before.py required the exact phase: the LLM fix passes it and the reference fails it (checked on 0.45.0, 1.2.4 and 2.5.0).</t>
         </is>
       </c>
       <c r="H254" s="67" t="n">
@@ -34144,14 +34076,14 @@
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="69" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="A255" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B255" s="67" t="inlineStr">
         <is>
-          <t>issue_985</t>
+          <t>issue_977</t>
         </is>
       </c>
       <c r="C255" s="67" t="inlineStr">
@@ -34162,19 +34094,11 @@
       <c r="D255" s="67" t="n">
         <v>23</v>
       </c>
-      <c r="E255" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError</t>
-        </is>
-      </c>
-      <c r="F255" s="67" t="inlineStr">
-        <is>
-          <t>AssertionError: Not equal to tolerance rtol=1e-07, atol=1e-12</t>
-        </is>
-      </c>
+      <c r="E255" s="67" t="n"/>
+      <c r="F255" s="67" t="n"/>
       <c r="G255" s="67" t="inlineStr">
         <is>
-          <t>The LLM replaced u1 with rz and set qc.global_phase = lam / 2, so the transpiled circuit uses only rx/ry/rz and equals U1(0.5) exactly, phase included, as the question asks. The current test requires the phase to be missing (determinant 1), following the answer's point that rotations alone cannot carry it. The team's earlier test_before.py required the exact phase: the LLM fix passes it and the reference fails it (checked on 0.45.0, 1.2.4 and 2.5.0).</t>
+          <t>Passed: the LLM replaced SparsePauliOp(Hamiltonian).to_operator() with SparsePauliOp.from_operator(Hamiltonian), the same call as the reference, and kept the variable name H_op. The updated test accepts any variable name.</t>
         </is>
       </c>
       <c r="H255" s="67" t="n">
@@ -34182,37 +34106,29 @@
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="70" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="A256" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B256" s="67" t="inlineStr">
         <is>
-          <t>issue_977</t>
+          <t>issue_994</t>
         </is>
       </c>
       <c r="C256" s="67" t="inlineStr">
         <is>
-          <t>0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3, 1.0.0, 1.0.1, 1.0.2, 1.1.0, 1.1.1, 1.1.2, 1.2.0, 1.2.1, 1.2.2, 1.2.4, 2.0.0, 2.2.0, 2.3.0, 2.4.0, 2.5.0</t>
+          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3</t>
         </is>
       </c>
       <c r="D256" s="67" t="n">
-        <v>23</v>
-      </c>
-      <c r="E256" s="67" t="inlineStr">
-        <is>
-          <t>KeyError</t>
-        </is>
-      </c>
-      <c r="F256" s="67" t="inlineStr">
-        <is>
-          <t>KeyError: 'op'</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="E256" s="67" t="n"/>
+      <c r="F256" s="67" t="n"/>
       <c r="G256" s="67" t="inlineStr">
         <is>
-          <t>The LLM used SparsePauliOp.from_operator(Hamiltonian), the same call as the reference, and kept the variable name H_op. The test reads the reference's variable name op. A test that accepts any variable name passes the LLM fix (checked on 0.45.0, 0.46.3, 1.0.0, 1.2.4 and 2.5.0) and still fails the buggy code.</t>
+          <t>Passed: the LLM added qc.save_statevector() so that get_statevector() works on the QasmSimulator. The updated test takes the statevector from either a variable or get_statevector().</t>
         </is>
       </c>
       <c r="H256" s="67" t="n">
@@ -34220,37 +34136,29 @@
       </c>
     </row>
     <row r="257">
-      <c r="A257" s="70" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="A257" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B257" s="67" t="inlineStr">
         <is>
-          <t>issue_994</t>
+          <t>issue_1035</t>
         </is>
       </c>
       <c r="C257" s="67" t="inlineStr">
         <is>
-          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3</t>
+          <t>0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3</t>
         </is>
       </c>
       <c r="D257" s="67" t="n">
-        <v>4</v>
-      </c>
-      <c r="E257" s="67" t="inlineStr">
-        <is>
-          <t>KeyError</t>
-        </is>
-      </c>
-      <c r="F257" s="67" t="inlineStr">
-        <is>
-          <t>KeyError: 'statevector'</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="E257" s="67" t="n"/>
+      <c r="F257" s="67" t="n"/>
       <c r="G257" s="67" t="inlineStr">
         <is>
-          <t>The LLM added qc.save_statevector() so that get_statevector() works on the QasmSimulator, and the script prints the Bell state. The test reads the reference's variable statevector and its snapshot data. A test that takes the statevector from either the variable or get_statevector() passes the LLM fix (checked on 0.25.0 and 0.25.3) and still fails the buggy code.</t>
+          <t>Passed: the LLM replaced the IBM Runtime service and session with Aer's local Estimator and the FakeManila noise model, which runs offline. The updated test accepts the result without a variable named result.</t>
         </is>
       </c>
       <c r="H257" s="67" t="n">
@@ -34258,41 +34166,33 @@
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="70" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="A258" s="68" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B258" s="67" t="inlineStr">
         <is>
-          <t>issue_1035</t>
+          <t>issue_772</t>
         </is>
       </c>
       <c r="C258" s="67" t="inlineStr">
         <is>
-          <t>0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3</t>
+          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3, 0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3</t>
         </is>
       </c>
       <c r="D258" s="67" t="n">
+        <v>12</v>
+      </c>
+      <c r="E258" s="67" t="n"/>
+      <c r="F258" s="67" t="n"/>
+      <c r="G258" s="67" t="inlineStr">
+        <is>
+          <t>The LLM passed the two register slices to append() as one combined qubit list (qr1[1:2] + qr2[0:3]), the same change the reference makes.</t>
+        </is>
+      </c>
+      <c r="H258" s="67" t="n">
         <v>8</v>
-      </c>
-      <c r="E258" s="67" t="inlineStr">
-        <is>
-          <t>KeyError</t>
-        </is>
-      </c>
-      <c r="F258" s="67" t="inlineStr">
-        <is>
-          <t>KeyError: 'result'</t>
-        </is>
-      </c>
-      <c r="G258" s="67" t="inlineStr">
-        <is>
-          <t>The LLM replaced the IBM Runtime service and session with Aer's local Estimator and the FakeManila noise model, which returns an expectation value near +1. The test reads the reference's variable result, but the LLM prints job.result().values without storing it. A test that also accepts job.result() passes the LLM fix (checked on 0.45.0 and 0.46.3) and still fails the buggy code.</t>
-        </is>
-      </c>
-      <c r="H258" s="67" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="259">
@@ -34303,22 +34203,22 @@
       </c>
       <c r="B259" s="67" t="inlineStr">
         <is>
-          <t>issue_772</t>
+          <t>issue_901</t>
         </is>
       </c>
       <c r="C259" s="67" t="inlineStr">
         <is>
-          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3, 0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3</t>
+          <t>0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3, 1.0.0, 1.0.1, 1.0.2, 1.1.0, 1.1.1, 1.1.2, 1.2.0, 1.2.1, 1.2.2, 1.2.4, 2.0.0</t>
         </is>
       </c>
       <c r="D259" s="67" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E259" s="67" t="n"/>
       <c r="F259" s="67" t="n"/>
       <c r="G259" s="67" t="inlineStr">
         <is>
-          <t>The LLM passed the two register slices to append() as one combined qubit list (qr1[1:2] + qr2[0:3]), the same change the reference makes.</t>
+          <t>The LLM replaced qc.s(0) with two T gates, which is exactly S, so the circuit transpiles into the H, T, CX basis. The reference keeps S and uses the Solovay-Kitaev pass instead.</t>
         </is>
       </c>
       <c r="H259" s="67" t="n">
@@ -34326,29 +34226,37 @@
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="68" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="A260" s="70" t="inlineStr">
+        <is>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="B260" s="67" t="inlineStr">
         <is>
-          <t>issue_901</t>
+          <t>issue_790</t>
         </is>
       </c>
       <c r="C260" s="67" t="inlineStr">
         <is>
-          <t>0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3, 1.0.0, 1.0.1, 1.0.2, 1.1.0, 1.1.1, 1.1.2, 1.2.0, 1.2.1, 1.2.2, 1.2.4, 2.0.0</t>
+          <t>0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3, 1.0.0, 1.0.1, 1.0.2, 1.1.0, 1.1.1, 1.1.2, 1.2.0, 1.2.1, 1.2.2, 1.2.4, 2.0.0, 2.2.0, 2.3.0, 2.4.0, 2.5.0</t>
         </is>
       </c>
       <c r="D260" s="67" t="n">
-        <v>19</v>
-      </c>
-      <c r="E260" s="67" t="n"/>
-      <c r="F260" s="67" t="n"/>
+        <v>23</v>
+      </c>
+      <c r="E260" s="67" t="inlineStr">
+        <is>
+          <t>TypeError</t>
+        </is>
+      </c>
+      <c r="F260" s="67" t="inlineStr">
+        <is>
+          <t>TypeError: unsupported operand type(s) for -: 'Pauli' and 'Pauli'</t>
+        </is>
+      </c>
       <c r="G260" s="67" t="inlineStr">
         <is>
-          <t>The LLM replaced qc.s(0) with two T gates, which is exactly S, so the circuit transpiles into the H, T, CX basis. The reference keeps S and uses the Solovay-Kitaev pass instead.</t>
+          <t>The LLM moved SuzukiTrotter.synthesize() onto each PauliEvolutionGate (the error the buggy code's comment points to) but kept (U * Z ^ Z) - (J * X ^ X) - (J * Y ^ Y); subtracting Pauli objects raises TypeError, exactly like the buggy code. The team's updated reference (6 Oct 2026) builds the same Hamiltonian with SparsePauliOp.from_list.</t>
         </is>
       </c>
       <c r="H260" s="67" t="n">
@@ -34363,30 +34271,30 @@
       </c>
       <c r="B261" s="67" t="inlineStr">
         <is>
-          <t>issue_790</t>
+          <t>issue_827</t>
         </is>
       </c>
       <c r="C261" s="67" t="inlineStr">
         <is>
-          <t>0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3, 1.0.0, 1.0.1, 1.0.2, 1.1.0, 1.1.1, 1.1.2, 1.2.0, 1.2.1, 1.2.2, 1.2.4, 2.0.0, 2.2.0, 2.3.0, 2.4.0, 2.5.0</t>
+          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3, 0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3</t>
         </is>
       </c>
       <c r="D261" s="67" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E261" s="67" t="inlineStr">
         <is>
-          <t>TypeError</t>
+          <t>ModuleNotFoundError</t>
         </is>
       </c>
       <c r="F261" s="67" t="inlineStr">
         <is>
-          <t>TypeError: unsupported operand type(s) for -: 'Pauli' and 'Pauli'</t>
+          <t>ModuleNotFoundError: No module named 'qiskit.backends'</t>
         </is>
       </c>
       <c r="G261" s="67" t="inlineStr">
         <is>
-          <t>The LLM moved SuzukiTrotter.synthesize() onto each PauliEvolutionGate (the error the buggy code's comment points to) but kept (U * Z ^ Z) - (J * X ^ X) - (J * Y ^ Y); subtracting Pauli objects raises TypeError, exactly like the buggy code. The team's updated reference (6 Oct 2026) builds the same Hamiltonian with SparsePauliOp.from_list.</t>
+          <t>The LLM replaced compile() with transpile() + assemble(), the reference's fix, but kept from qiskit.backends.jobstatus import JOB_FINAL_STATES; qiskit.backends no longer exists. With only that import changed to qiskit.providers.jobstatus the fix passes (checked on 0.25.0, 0.45.0 and 0.46.3).</t>
         </is>
       </c>
       <c r="H261" s="67" t="n">
@@ -34401,30 +34309,30 @@
       </c>
       <c r="B262" s="67" t="inlineStr">
         <is>
-          <t>issue_827</t>
+          <t>issue_858</t>
         </is>
       </c>
       <c r="C262" s="67" t="inlineStr">
         <is>
-          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3, 0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3</t>
+          <t>0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3</t>
         </is>
       </c>
       <c r="D262" s="67" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E262" s="67" t="inlineStr">
         <is>
-          <t>ModuleNotFoundError</t>
+          <t>OfflineAccessDenied</t>
         </is>
       </c>
       <c r="F262" s="67" t="inlineStr">
         <is>
-          <t>ModuleNotFoundError: No module named 'qiskit.backends'</t>
+          <t>OfflineAccessDenied: Offline snapshot fixture forbids IBMQ.load_account</t>
         </is>
       </c>
       <c r="G262" s="67" t="inlineStr">
         <is>
-          <t>The LLM replaced compile() with transpile() + assemble(), the reference's fix, but kept from qiskit.backends.jobstatus import JOB_FINAL_STATES; qiskit.backends no longer exists. With only that import changed to qiskit.providers.jobstatus the fix passes (checked on 0.25.0, 0.45.0 and 0.46.3).</t>
+          <t>The LLM switched to the FakeOslo snapshot but kept the unused provider = IBMQ.load_account(), which needs an IBM account online; the offline test blocks it. With that line removed it still crashes: FakeOslo has no properties() method (checked on 0.45.0 and 0.46.3). The reference reads backend.qubit_properties().</t>
         </is>
       </c>
       <c r="H262" s="67" t="n">
@@ -34439,71 +34347,33 @@
       </c>
       <c r="B263" s="67" t="inlineStr">
         <is>
-          <t>issue_858</t>
+          <t>issue_921</t>
         </is>
       </c>
       <c r="C263" s="67" t="inlineStr">
         <is>
-          <t>0.45.0, 0.45.1, 0.45.2, 0.45.3, 0.46.0, 0.46.1, 0.46.2, 0.46.3</t>
+          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3</t>
         </is>
       </c>
       <c r="D263" s="67" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E263" s="67" t="inlineStr">
         <is>
-          <t>OfflineAccessDenied</t>
+          <t>ImportError</t>
         </is>
       </c>
       <c r="F263" s="67" t="inlineStr">
         <is>
-          <t>OfflineAccessDenied: Offline snapshot fixture forbids IBMQ.load_account</t>
+          <t>ImportError: cannot import name 'run_algorithm' from 'qiskit.aqua' (C:\qiskit_envs\q0250\lib\site-packages\qiskit\aqua\__init__.py)</t>
         </is>
       </c>
       <c r="G263" s="67" t="inlineStr">
         <is>
-          <t>The LLM switched to the FakeOslo snapshot but kept the unused provider = IBMQ.load_account(), which needs an IBM account online; the offline test blocks it. With that line removed it still crashes: FakeOslo has no properties() method (checked on 0.45.0 and 0.46.3). The reference reads backend.qubit_properties().</t>
+          <t>The LLM returned the buggy code unchanged, without the required '# NO BUG:' line, so run_algorithm is still missing from qiskit.aqua (ImportError), exactly like the buggy code. The reference calls ExactEigensolver(qubitOp, k=1).run().</t>
         </is>
       </c>
       <c r="H263" s="67" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" s="70" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="B264" s="67" t="inlineStr">
-        <is>
-          <t>issue_921</t>
-        </is>
-      </c>
-      <c r="C264" s="67" t="inlineStr">
-        <is>
-          <t>0.25.0, 0.25.1, 0.25.2, 0.25.3</t>
-        </is>
-      </c>
-      <c r="D264" s="67" t="n">
-        <v>4</v>
-      </c>
-      <c r="E264" s="67" t="inlineStr">
-        <is>
-          <t>ImportError</t>
-        </is>
-      </c>
-      <c r="F264" s="67" t="inlineStr">
-        <is>
-          <t>ImportError: cannot import name 'run_algorithm' from 'qiskit.aqua' (C:\qiskit_envs\q0250\lib\site-packages\qiskit\aqua\__init__.py)</t>
-        </is>
-      </c>
-      <c r="G264" s="67" t="inlineStr">
-        <is>
-          <t>The LLM returned the buggy code unchanged, without the required '# NO BUG:' line, so run_algorithm is still missing from qiskit.aqua (ImportError), exactly like the buggy code. The reference calls ExactEigensolver(qubitOp, k=1).run().</t>
-        </is>
-      </c>
-      <c r="H264" s="67" t="n">
         <v>8</v>
       </c>
     </row>
@@ -34835,7 +34705,7 @@
       </c>
       <c r="B10" s="22" t="inlineStr">
         <is>
-          <t>Over-specific</t>
+          <t>Over-specific in the old test.py; replaced by the updated test, now the case's test.py (9 Oct 2026)</t>
         </is>
       </c>
       <c r="C10" s="23" t="inlineStr">
@@ -34860,7 +34730,7 @@
       </c>
       <c r="G10" s="24" t="inlineStr">
         <is>
-          <t>This is the only reason the LLM fails. Its fix uses [n-1-i, 3, ..., 8] and every gate matrix is correct (checked separately), but the qubit-list check fails first on all 23 versions. A test that accepted either control order would pass it.</t>
+          <t>On 9 Oct 2026 the case's test.py was replaced by an updated version, which drops this requirement and still fails the buggy code and passes the reference on every version. With the updated test the LLM fix passes on every version.</t>
         </is>
       </c>
       <c r="H10" s="25">
@@ -35285,7 +35155,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>Over-specific</t>
+          <t>Over-specific in the old test.py; replaced by the updated test, now the case's test.py (9 Oct 2026)</t>
         </is>
       </c>
       <c r="C20" s="23" t="inlineStr">
@@ -35310,7 +35180,7 @@
       </c>
       <c r="G20" s="24" t="inlineStr">
         <is>
-          <t>This is the only reason the LLM fails. FakeYorktown (5 qubits) fixes the error and gives 933 of 1024 shots as '00'/'11' (91%); every other check passes. A test that allowed a little noise, or only checked the qubit count and the Bell state, would pass it. FAIL on all 12 versions.</t>
+          <t>On 9 Oct 2026 the case's test.py was replaced by an updated version, which drops this requirement and still fails the buggy code and passes the reference on every version. With the updated test the LLM fix passes on every version.</t>
         </is>
       </c>
       <c r="H20" s="25">
@@ -35465,7 +35335,7 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>Over-specific</t>
+          <t>Over-specific in the old test.py; replaced by the updated test, now the case's test.py (9 Oct 2026)</t>
         </is>
       </c>
       <c r="C24" s="23" t="inlineStr">
@@ -35490,7 +35360,7 @@
       </c>
       <c r="G24" s="24" t="inlineStr">
         <is>
-          <t>This is the only reason the LLM fails. QuantumCircuit(a, *v, b) passes every register check; without the unitary check it passes (checked on 5 versions) and the buggy code still fails. FAIL on all 27 versions.</t>
+          <t>On 9 Oct 2026 the case's test.py was replaced by an updated version, which drops this requirement and still fails the buggy code and passes the reference on every version. With the updated test the LLM fix passes on every version.</t>
         </is>
       </c>
       <c r="H24" s="25">
@@ -35510,7 +35380,7 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>Over-specific</t>
+          <t>Over-specific in the old test.py; replaced by the updated test, now the case's test.py (9 Oct 2026)</t>
         </is>
       </c>
       <c r="C25" s="23" t="inlineStr">
@@ -35535,7 +35405,7 @@
       </c>
       <c r="G25" s="24" t="inlineStr">
         <is>
-          <t>This is the only reason the LLM fails (KeyError: 'qc'). A test that checks the executed result (success, 1 experiment, 2 qubits, 2 memory slots) passes the LLM fix on 0.25.0, 0.45.0 and 0.46.3 and still fails the buggy code. ERROR on all 12 versions.</t>
+          <t>On 9 Oct 2026 the case's test.py was replaced by an updated version, which drops this requirement and still fails the buggy code and passes the reference on every version. With the updated test the LLM fix passes on every version.</t>
         </is>
       </c>
       <c r="H25" s="25">
@@ -35555,7 +35425,7 @@
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>Borderline (count format)</t>
+          <t>Borderline (count format) in the old test.py; replaced by the updated test, now the case's test.py (9 Oct 2026)</t>
         </is>
       </c>
       <c r="C26" s="23" t="inlineStr">
@@ -35580,7 +35450,7 @@
       </c>
       <c r="G26" s="24" t="inlineStr">
         <is>
-          <t>This is the only reason the LLM fails. Its statistics are correct GHZ statistics; a test that ignores the unused register passes it on 0.45.0 and 0.46.3. Still, leaving 3 unused classical bits is sloppier than the reference. FAIL on all 8 versions.</t>
+          <t>On 9 Oct 2026 the case's test.py was replaced by an updated version, which drops this requirement and still fails the buggy code and passes the reference on every version. With the updated test the LLM fix passes on every version.</t>
         </is>
       </c>
       <c r="H26" s="25">
@@ -35645,7 +35515,7 @@
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
-          <t>Over-specific</t>
+          <t>Over-specific in the old test.py; replaced by the updated test, now the case's test.py (9 Oct 2026)</t>
         </is>
       </c>
       <c r="C28" s="23" t="inlineStr">
@@ -35670,7 +35540,7 @@
       </c>
       <c r="G28" s="24" t="inlineStr">
         <is>
-          <t>This is the only reason the LLM fails. a = job.result().get_counts() is the same call as the reference; a test that accepts any variable name and the script's own shot count passes it on 0.45.1 and 0.46.2. FAIL on both versions.</t>
+          <t>On 9 Oct 2026 the case's test.py was replaced by an updated version, which drops this requirement and still fails the buggy code and passes the reference on every version. With the updated test the LLM fix passes on every version.</t>
         </is>
       </c>
       <c r="H28" s="25">
@@ -35690,7 +35560,7 @@
       </c>
       <c r="B29" s="22" t="inlineStr">
         <is>
-          <t>Over-specific</t>
+          <t>Over-specific in the old test.py; replaced by the updated test, now the case's test.py (9 Oct 2026)</t>
         </is>
       </c>
       <c r="C29" s="23" t="inlineStr">
@@ -35715,7 +35585,7 @@
       </c>
       <c r="G29" s="24" t="inlineStr">
         <is>
-          <t>This is the only reason the LLM fails. It transpiles exactly like the answer; a test that ignores the unused register and the variable name passes it on 0.45.0 and 0.45.1. FAIL on both versions.</t>
+          <t>On 9 Oct 2026 the case's test.py was replaced by an updated version, which drops this requirement and still fails the buggy code and passes the reference on every version. With the updated test the LLM fix passes on every version.</t>
         </is>
       </c>
       <c r="H29" s="25">
@@ -35735,7 +35605,7 @@
       </c>
       <c r="B30" s="22" t="inlineStr">
         <is>
-          <t>Over-specific (print format)</t>
+          <t>Over-specific (print format) in the old test.py; replaced by the updated test, now the case's test.py (9 Oct 2026)</t>
         </is>
       </c>
       <c r="C30" s="23" t="inlineStr">
@@ -35760,7 +35630,7 @@
       </c>
       <c r="G30" s="24" t="inlineStr">
         <is>
-          <t>This is the only reason the LLM fails. It prints each qubit's index with find_bit (and keeps the original 'qargs :' line with Qubit objects); a test that reads the indices in either format passes it on 0.45.0, 1.0.0, 1.2.4 and 2.5.0. ERROR on all 23 versions.</t>
+          <t>On 9 Oct 2026 the case's test.py was replaced by an updated version, which drops this requirement and still fails the buggy code and passes the reference on every version. With the updated test the LLM fix passes on every version.</t>
         </is>
       </c>
       <c r="H30" s="25">
@@ -35780,7 +35650,7 @@
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>Over-specific (operator type)</t>
+          <t>Over-specific (operator type) in the old test.py; replaced by the updated test, now the case's test.py (9 Oct 2026)</t>
         </is>
       </c>
       <c r="C31" s="23" t="inlineStr">
@@ -35805,7 +35675,7 @@
       </c>
       <c r="G31" s="24" t="inlineStr">
         <is>
-          <t>This is the only reason the LLM fails. Its opflow projector has the right matrix and eigenvalues; a test that accepts either operator type passes it on 0.25.0, 0.45.0 and 0.46.3. ERROR on all 12 versions.</t>
+          <t>On 9 Oct 2026 the case's test.py was replaced by an updated version, which drops this requirement and still fails the buggy code and passes the reference on every version. With the updated test the LLM fix passes on every version.</t>
         </is>
       </c>
       <c r="H31" s="25">
@@ -35870,7 +35740,7 @@
       </c>
       <c r="B33" s="22" t="inlineStr">
         <is>
-          <t>Over-specific (variable name)</t>
+          <t>Over-specific (variable name) in the old test.py; replaced by the updated test, now the case's test.py (9 Oct 2026)</t>
         </is>
       </c>
       <c r="C33" s="23" t="inlineStr">
@@ -35895,7 +35765,7 @@
       </c>
       <c r="G33" s="24" t="inlineStr">
         <is>
-          <t>This is the only reason the LLM fails. H_op = SparsePauliOp.from_operator(Hamiltonian) is the same call as the reference; a test that accepts any variable name passes it on 0.45.0, 0.46.3, 1.0.0, 1.2.4 and 2.5.0. ERROR on all 23 versions.</t>
+          <t>On 9 Oct 2026 the case's test.py was replaced by an updated version, which drops this requirement and still fails the buggy code and passes the reference on every version. With the updated test the LLM fix passes on every version.</t>
         </is>
       </c>
       <c r="H33" s="25">
@@ -35915,7 +35785,7 @@
       </c>
       <c r="B34" s="22" t="inlineStr">
         <is>
-          <t>Over-specific (snapshot method)</t>
+          <t>Over-specific (snapshot method) in the old test.py; replaced by the updated test, now the case's test.py (9 Oct 2026)</t>
         </is>
       </c>
       <c r="C34" s="23" t="inlineStr">
@@ -35940,7 +35810,7 @@
       </c>
       <c r="G34" s="24" t="inlineStr">
         <is>
-          <t>This is the only reason the LLM fails. A test that takes the statevector from either the variable or get_statevector() passes it on 0.25.0 and 0.25.3. ERROR on all 4 versions.</t>
+          <t>On 9 Oct 2026 the case's test.py was replaced by an updated version, which drops this requirement and still fails the buggy code and passes the reference on every version. With the updated test the LLM fix passes on every version.</t>
         </is>
       </c>
       <c r="H34" s="25">
@@ -35960,7 +35830,7 @@
       </c>
       <c r="B35" s="22" t="inlineStr">
         <is>
-          <t>Over-specific (variable name)</t>
+          <t>Over-specific (variable name) in the old test.py; replaced by the updated test, now the case's test.py (9 Oct 2026)</t>
         </is>
       </c>
       <c r="C35" s="23" t="inlineStr">
@@ -35985,7 +35855,7 @@
       </c>
       <c r="G35" s="24" t="inlineStr">
         <is>
-          <t>This is the only reason the LLM fails. Its Aer Estimator with FakeManila's noise model runs offline; a test that also accepts job.result() passes it on 0.45.0 and 0.46.3. ERROR on all 8 versions.</t>
+          <t>On 9 Oct 2026 the case's test.py was replaced by an updated version, which drops this requirement and still fails the buggy code and passes the reference on every version. With the updated test the LLM fix passes on every version.</t>
         </is>
       </c>
       <c r="H35" s="25">
@@ -36098,7 +35968,7 @@
     <row r="40" ht="240" customHeight="1" s="35">
       <c r="A40" s="34" t="inlineStr">
         <is>
-          <t>issue_061's old test was over-specific; the team's updated test_new.py fixes that and the LLM fix now passes 15/15. issue_096 still asks for more than the question (exact '[default]' content and exact os.system command), but the LLM fix would fail a fair test too because it skips the IPython step. The extra checks in 021_se, 034 and 058_se are fair and did not change any result. Batch 2: issue_189 is over-specific. It only accepts the Stack Overflow answer's control order, and that is the only reason the LLM fix fails. The extra checks in issue_174, issue_233, issue_295 and issue_315 are fair; the LLM failures in 174, 233 and 315 are its own mistakes. Batch 3: issue_453 is over-specific (it requires the answer's compose_with_auto_ancillas helper by name), though the LLM fix also misses the automatic-ancilla part of the question. issue_415's last check pins a global phase, but the LLM fails an earlier fair check. The extra checks in issue_344, issue_369 and issue_436 are fair. Batch 4: issue_622 is over-specific. It requires noise-free counts, and that is the only reason the LLM's FakeYorktown fix fails. The extra checks in issue_565, issue_596 and issue_635 are fair; the LLM failures in 565 and 635 are its own mistakes. Batch 5: issue_671 and issue_775 are over-specific. 671 checks the unitary of the answer's example gates and 775 requires a variable named qc; that is the only reason the LLM fails both, and relaxed tests pass the LLM fixes. issue_747 is borderline: the test requires the exact keys '000'/'111', and the LLM's measure_all() adds a second register. issue_769 needs the answer's function name, but the LLM fix would fail a fair test too. Batch 6: issue_810, issue_886, issue_911 and issue_944 are over-specific (a variable name and shot count, an exact count key and variable name, an exact print format, and an attribute only the reference's operator type has); in all four, relaxed tests pass the LLM fix and still fail the buggy code. issue_877 pins 27 qubits, but the LLM's empty noise model would fail a fair test too. Batch 7: issue_977, issue_994 and issue_1035 are over-specific (a variable name, the reference's snapshot method, and a variable name); in all three, relaxed tests pass the LLM fix and still fail the buggy code. issue_985 is debatable: the test requires the phase to be dropped, while the LLM keeps it exactly with global_phase (and passes the team's earlier test). issue_958 needs the reference's extra circuit qc2, but the LLM fix fails the fair check too. Batch 8: all 6 tests are fair. issue_790's reference fix was updated by the team on 6 Oct 2026 and now passes its test, and issue_827 got its test the same day. Relaxed tests run on every version (6 Oct 2026): for all 11 over-specific cases the relaxed test fails the buggy code, passes the reference and passes the LLM fix on every version; see the Relaxed Tests sheet.</t>
+          <t>issue_061's old test was over-specific; the team's updated test_new.py fixes that and the LLM fix now passes 15/15. issue_096 still asks for more than the question (exact '[default]' content and exact os.system command), but the LLM fix would fail a fair test too because it skips the IPython step. The extra checks in 021_se, 034 and 058_se are fair and did not change any result. Batch 2: issue_189 is over-specific. It only accepts the Stack Overflow answer's control order, and that is the only reason the LLM fix fails. The extra checks in issue_174, issue_233, issue_295 and issue_315 are fair; the LLM failures in 174, 233 and 315 are its own mistakes. Batch 3: issue_453 is over-specific (it requires the answer's compose_with_auto_ancillas helper by name), though the LLM fix also misses the automatic-ancilla part of the question. issue_415's last check pins a global phase, but the LLM fails an earlier fair check. The extra checks in issue_344, issue_369 and issue_436 are fair. Batch 4: issue_622 is over-specific. It requires noise-free counts, and that is the only reason the LLM's FakeYorktown fix fails. The extra checks in issue_565, issue_596 and issue_635 are fair; the LLM failures in 565 and 635 are its own mistakes. Batch 5: issue_671 and issue_775 are over-specific. 671 checks the unitary of the answer's example gates and 775 requires a variable named qc; that is the only reason the LLM failed both, and both fixes pass the updated tests. issue_747 is borderline: the test requires the exact keys '000'/'111', and the LLM's measure_all() adds a second register. issue_769 needs the answer's function name, but the LLM fix would fail a fair test too. Batch 6: issue_810, issue_886, issue_911 and issue_944 are over-specific (a variable name and shot count, an exact count key and variable name, an exact print format, and an attribute only the reference's operator type has); the LLM fix passes all four updated tests. issue_877 pins 27 qubits, but the LLM's empty noise model would fail a fair test too. Batch 7: issue_977, issue_994 and issue_1035 are over-specific (a variable name, the reference's snapshot method, and a variable name); the LLM fix passes all three updated tests. issue_985 is debatable: the test requires the phase to be dropped, while the LLM keeps it exactly with global_phase (and passes the team's earlier test). issue_958 needs the reference's extra circuit qc2, but the LLM fix fails the fair check too. Batch 8: all 6 tests are fair. issue_790's reference fix was updated by the team on 6 Oct 2026 and now passes its test, and issue_827 got its test the same day. Update 9 Oct 2026: the 12 over-specific tests (189, 622, 671, 747, 775, 810, 886, 911, 944, 977, 994, 1035) were replaced by the updated tests (each case's test.py now holds the updated version), which fail the buggy code and pass the reference on every version; every model was retested on them, and the LLM fix passes all 12 on every version.</t>
         </is>
       </c>
     </row>
@@ -36110,730 +35980,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" style="35" min="1" max="1"/>
-    <col width="7" customWidth="1" style="35" min="2" max="2"/>
-    <col width="11" customWidth="1" style="35" min="3" max="3"/>
-    <col width="22" customWidth="1" style="35" min="4" max="4"/>
-    <col width="10" customWidth="1" style="35" min="5" max="5"/>
-    <col width="12" customWidth="1" style="35" min="6" max="6"/>
-    <col width="14" customWidth="1" style="35" min="7" max="7"/>
-    <col width="16" customWidth="1" style="35" min="8" max="8"/>
-    <col width="16" customWidth="1" style="35" min="9" max="9"/>
-    <col width="18" customWidth="1" style="35" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="60" t="inlineStr">
-        <is>
-          <t>Relaxed tests on every version (6 Oct 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="75" customHeight="1" s="35">
-      <c r="A2" s="71" t="inlineStr">
-        <is>
-          <t>Each over-specific test was rewritten without the detail only the reference has (a variable name, print format, operator type, control order, noise-free counts or example gates). A relaxed test counts as valid on a version if it still fails buggy.py and passes fixed.py. issue_747 (borderline) uses a test that ignores the extra measure_all() register; issue_985 (debatable) uses the team's earlier test_before.py, which requires the exact U1 phase, so the reference is expected to fail it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="54" t="inlineStr">
-        <is>
-          <t>Case</t>
-        </is>
-      </c>
-      <c r="B4" s="54" t="inlineStr">
-        <is>
-          <t>Batch</t>
-        </is>
-      </c>
-      <c r="C4" s="54" t="inlineStr">
-        <is>
-          <t>Kind</t>
-        </is>
-      </c>
-      <c r="D4" s="54" t="inlineStr">
-        <is>
-          <t>Relaxed test</t>
-        </is>
-      </c>
-      <c r="E4" s="54" t="inlineStr">
-        <is>
-          <t>Versions</t>
-        </is>
-      </c>
-      <c r="F4" s="54" t="inlineStr">
-        <is>
-          <t>Relaxed test valid</t>
-        </is>
-      </c>
-      <c r="G4" s="54" t="inlineStr">
-        <is>
-          <t>Buggy</t>
-        </is>
-      </c>
-      <c r="H4" s="54" t="inlineStr">
-        <is>
-          <t>Fixed (reference)</t>
-        </is>
-      </c>
-      <c r="I4" s="54" t="inlineStr">
-        <is>
-          <t>LLM fix (relaxed)</t>
-        </is>
-      </c>
-      <c r="J4" s="54" t="inlineStr">
-        <is>
-          <t>LLM fix (official test)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="67" t="inlineStr">
-        <is>
-          <t>issue_189</t>
-        </is>
-      </c>
-      <c r="B5" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="C5" s="67" t="inlineStr">
-        <is>
-          <t>strict</t>
-        </is>
-      </c>
-      <c r="D5" s="67" t="inlineStr">
-        <is>
-          <t>189_relaxed_test.py</t>
-        </is>
-      </c>
-      <c r="E5" s="67" t="n">
-        <v>23</v>
-      </c>
-      <c r="F5" s="67" t="inlineStr">
-        <is>
-          <t>23 / 23</t>
-        </is>
-      </c>
-      <c r="G5" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 23</t>
-        </is>
-      </c>
-      <c r="H5" s="67" t="inlineStr">
-        <is>
-          <t>PASS 23</t>
-        </is>
-      </c>
-      <c r="I5" s="68" t="inlineStr">
-        <is>
-          <t>PASS 23</t>
-        </is>
-      </c>
-      <c r="J5" s="67" t="inlineStr">
-        <is>
-          <t>FAIL 23</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="67" t="inlineStr">
-        <is>
-          <t>issue_622</t>
-        </is>
-      </c>
-      <c r="B6" s="67" t="n">
-        <v>4</v>
-      </c>
-      <c r="C6" s="67" t="inlineStr">
-        <is>
-          <t>strict</t>
-        </is>
-      </c>
-      <c r="D6" s="67" t="inlineStr">
-        <is>
-          <t>622_relaxed_test.py</t>
-        </is>
-      </c>
-      <c r="E6" s="67" t="n">
-        <v>12</v>
-      </c>
-      <c r="F6" s="67" t="inlineStr">
-        <is>
-          <t>12 / 12</t>
-        </is>
-      </c>
-      <c r="G6" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 12</t>
-        </is>
-      </c>
-      <c r="H6" s="67" t="inlineStr">
-        <is>
-          <t>PASS 12</t>
-        </is>
-      </c>
-      <c r="I6" s="68" t="inlineStr">
-        <is>
-          <t>PASS 12</t>
-        </is>
-      </c>
-      <c r="J6" s="67" t="inlineStr">
-        <is>
-          <t>FAIL 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="67" t="inlineStr">
-        <is>
-          <t>issue_671</t>
-        </is>
-      </c>
-      <c r="B7" s="67" t="n">
-        <v>5</v>
-      </c>
-      <c r="C7" s="67" t="inlineStr">
-        <is>
-          <t>strict</t>
-        </is>
-      </c>
-      <c r="D7" s="67" t="inlineStr">
-        <is>
-          <t>671_relaxed_test.py</t>
-        </is>
-      </c>
-      <c r="E7" s="67" t="n">
-        <v>27</v>
-      </c>
-      <c r="F7" s="67" t="inlineStr">
-        <is>
-          <t>27 / 27</t>
-        </is>
-      </c>
-      <c r="G7" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 27</t>
-        </is>
-      </c>
-      <c r="H7" s="67" t="inlineStr">
-        <is>
-          <t>PASS 27</t>
-        </is>
-      </c>
-      <c r="I7" s="68" t="inlineStr">
-        <is>
-          <t>PASS 27</t>
-        </is>
-      </c>
-      <c r="J7" s="67" t="inlineStr">
-        <is>
-          <t>FAIL 27</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="67" t="inlineStr">
-        <is>
-          <t>issue_775</t>
-        </is>
-      </c>
-      <c r="B8" s="67" t="n">
-        <v>5</v>
-      </c>
-      <c r="C8" s="67" t="inlineStr">
-        <is>
-          <t>strict</t>
-        </is>
-      </c>
-      <c r="D8" s="67" t="inlineStr">
-        <is>
-          <t>775_relaxed_test.py</t>
-        </is>
-      </c>
-      <c r="E8" s="67" t="n">
-        <v>12</v>
-      </c>
-      <c r="F8" s="67" t="inlineStr">
-        <is>
-          <t>12 / 12</t>
-        </is>
-      </c>
-      <c r="G8" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 12</t>
-        </is>
-      </c>
-      <c r="H8" s="67" t="inlineStr">
-        <is>
-          <t>PASS 12</t>
-        </is>
-      </c>
-      <c r="I8" s="68" t="inlineStr">
-        <is>
-          <t>PASS 12</t>
-        </is>
-      </c>
-      <c r="J8" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="67" t="inlineStr">
-        <is>
-          <t>issue_810</t>
-        </is>
-      </c>
-      <c r="B9" s="67" t="n">
-        <v>6</v>
-      </c>
-      <c r="C9" s="67" t="inlineStr">
-        <is>
-          <t>strict</t>
-        </is>
-      </c>
-      <c r="D9" s="67" t="inlineStr">
-        <is>
-          <t>810_relaxed_test.py</t>
-        </is>
-      </c>
-      <c r="E9" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="F9" s="67" t="inlineStr">
-        <is>
-          <t>2 / 2</t>
-        </is>
-      </c>
-      <c r="G9" s="67" t="inlineStr">
-        <is>
-          <t>FAIL 2</t>
-        </is>
-      </c>
-      <c r="H9" s="67" t="inlineStr">
-        <is>
-          <t>PASS 2</t>
-        </is>
-      </c>
-      <c r="I9" s="68" t="inlineStr">
-        <is>
-          <t>PASS 2</t>
-        </is>
-      </c>
-      <c r="J9" s="67" t="inlineStr">
-        <is>
-          <t>FAIL 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="67" t="inlineStr">
-        <is>
-          <t>issue_886</t>
-        </is>
-      </c>
-      <c r="B10" s="67" t="n">
-        <v>6</v>
-      </c>
-      <c r="C10" s="67" t="inlineStr">
-        <is>
-          <t>strict</t>
-        </is>
-      </c>
-      <c r="D10" s="67" t="inlineStr">
-        <is>
-          <t>886_relaxed_test.py</t>
-        </is>
-      </c>
-      <c r="E10" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" s="67" t="inlineStr">
-        <is>
-          <t>2 / 2</t>
-        </is>
-      </c>
-      <c r="G10" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 2</t>
-        </is>
-      </c>
-      <c r="H10" s="67" t="inlineStr">
-        <is>
-          <t>PASS 2</t>
-        </is>
-      </c>
-      <c r="I10" s="68" t="inlineStr">
-        <is>
-          <t>PASS 2</t>
-        </is>
-      </c>
-      <c r="J10" s="67" t="inlineStr">
-        <is>
-          <t>FAIL 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="67" t="inlineStr">
-        <is>
-          <t>issue_911</t>
-        </is>
-      </c>
-      <c r="B11" s="67" t="n">
-        <v>6</v>
-      </c>
-      <c r="C11" s="67" t="inlineStr">
-        <is>
-          <t>strict</t>
-        </is>
-      </c>
-      <c r="D11" s="67" t="inlineStr">
-        <is>
-          <t>911_relaxed_test.py</t>
-        </is>
-      </c>
-      <c r="E11" s="67" t="n">
-        <v>23</v>
-      </c>
-      <c r="F11" s="67" t="inlineStr">
-        <is>
-          <t>23 / 23</t>
-        </is>
-      </c>
-      <c r="G11" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 23</t>
-        </is>
-      </c>
-      <c r="H11" s="67" t="inlineStr">
-        <is>
-          <t>PASS 23</t>
-        </is>
-      </c>
-      <c r="I11" s="68" t="inlineStr">
-        <is>
-          <t>PASS 23</t>
-        </is>
-      </c>
-      <c r="J11" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 23</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="67" t="inlineStr">
-        <is>
-          <t>issue_944</t>
-        </is>
-      </c>
-      <c r="B12" s="67" t="n">
-        <v>6</v>
-      </c>
-      <c r="C12" s="67" t="inlineStr">
-        <is>
-          <t>strict</t>
-        </is>
-      </c>
-      <c r="D12" s="67" t="inlineStr">
-        <is>
-          <t>944_relaxed_test.py</t>
-        </is>
-      </c>
-      <c r="E12" s="67" t="n">
-        <v>12</v>
-      </c>
-      <c r="F12" s="67" t="inlineStr">
-        <is>
-          <t>12 / 12</t>
-        </is>
-      </c>
-      <c r="G12" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 12</t>
-        </is>
-      </c>
-      <c r="H12" s="67" t="inlineStr">
-        <is>
-          <t>PASS 12</t>
-        </is>
-      </c>
-      <c r="I12" s="68" t="inlineStr">
-        <is>
-          <t>PASS 12</t>
-        </is>
-      </c>
-      <c r="J12" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="67" t="inlineStr">
-        <is>
-          <t>issue_977</t>
-        </is>
-      </c>
-      <c r="B13" s="67" t="n">
-        <v>7</v>
-      </c>
-      <c r="C13" s="67" t="inlineStr">
-        <is>
-          <t>strict</t>
-        </is>
-      </c>
-      <c r="D13" s="67" t="inlineStr">
-        <is>
-          <t>977_relaxed_test.py</t>
-        </is>
-      </c>
-      <c r="E13" s="67" t="n">
-        <v>23</v>
-      </c>
-      <c r="F13" s="67" t="inlineStr">
-        <is>
-          <t>23 / 23</t>
-        </is>
-      </c>
-      <c r="G13" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 23</t>
-        </is>
-      </c>
-      <c r="H13" s="67" t="inlineStr">
-        <is>
-          <t>PASS 23</t>
-        </is>
-      </c>
-      <c r="I13" s="68" t="inlineStr">
-        <is>
-          <t>PASS 23</t>
-        </is>
-      </c>
-      <c r="J13" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 23</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="67" t="inlineStr">
-        <is>
-          <t>issue_994</t>
-        </is>
-      </c>
-      <c r="B14" s="67" t="n">
-        <v>7</v>
-      </c>
-      <c r="C14" s="67" t="inlineStr">
-        <is>
-          <t>strict</t>
-        </is>
-      </c>
-      <c r="D14" s="67" t="inlineStr">
-        <is>
-          <t>994_relaxed_test.py</t>
-        </is>
-      </c>
-      <c r="E14" s="67" t="n">
-        <v>4</v>
-      </c>
-      <c r="F14" s="67" t="inlineStr">
-        <is>
-          <t>4 / 4</t>
-        </is>
-      </c>
-      <c r="G14" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 4</t>
-        </is>
-      </c>
-      <c r="H14" s="67" t="inlineStr">
-        <is>
-          <t>PASS 4</t>
-        </is>
-      </c>
-      <c r="I14" s="68" t="inlineStr">
-        <is>
-          <t>PASS 4</t>
-        </is>
-      </c>
-      <c r="J14" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="67" t="inlineStr">
-        <is>
-          <t>issue_1035</t>
-        </is>
-      </c>
-      <c r="B15" s="67" t="n">
-        <v>7</v>
-      </c>
-      <c r="C15" s="67" t="inlineStr">
-        <is>
-          <t>strict</t>
-        </is>
-      </c>
-      <c r="D15" s="67" t="inlineStr">
-        <is>
-          <t>1035_relaxed_test.py</t>
-        </is>
-      </c>
-      <c r="E15" s="67" t="n">
-        <v>8</v>
-      </c>
-      <c r="F15" s="67" t="inlineStr">
-        <is>
-          <t>8 / 8</t>
-        </is>
-      </c>
-      <c r="G15" s="67" t="inlineStr">
-        <is>
-          <t>FAIL 8</t>
-        </is>
-      </c>
-      <c r="H15" s="67" t="inlineStr">
-        <is>
-          <t>PASS 8</t>
-        </is>
-      </c>
-      <c r="I15" s="68" t="inlineStr">
-        <is>
-          <t>PASS 8</t>
-        </is>
-      </c>
-      <c r="J15" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 8</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="67" t="inlineStr">
-        <is>
-          <t>issue_747</t>
-        </is>
-      </c>
-      <c r="B16" s="67" t="n">
-        <v>5</v>
-      </c>
-      <c r="C16" s="67" t="inlineStr">
-        <is>
-          <t>borderline</t>
-        </is>
-      </c>
-      <c r="D16" s="67" t="inlineStr">
-        <is>
-          <t>747_relaxed_test.py</t>
-        </is>
-      </c>
-      <c r="E16" s="67" t="n">
-        <v>8</v>
-      </c>
-      <c r="F16" s="67" t="inlineStr">
-        <is>
-          <t>8 / 8</t>
-        </is>
-      </c>
-      <c r="G16" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 8</t>
-        </is>
-      </c>
-      <c r="H16" s="67" t="inlineStr">
-        <is>
-          <t>PASS 8</t>
-        </is>
-      </c>
-      <c r="I16" s="68" t="inlineStr">
-        <is>
-          <t>PASS 8</t>
-        </is>
-      </c>
-      <c r="J16" s="67" t="inlineStr">
-        <is>
-          <t>FAIL 8</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="67" t="inlineStr">
-        <is>
-          <t>issue_985</t>
-        </is>
-      </c>
-      <c r="B17" s="67" t="n">
-        <v>7</v>
-      </c>
-      <c r="C17" s="67" t="inlineStr">
-        <is>
-          <t>debatable</t>
-        </is>
-      </c>
-      <c r="D17" s="67" t="inlineStr">
-        <is>
-          <t>test_before.py</t>
-        </is>
-      </c>
-      <c r="E17" s="67" t="n">
-        <v>23</v>
-      </c>
-      <c r="F17" s="67" t="inlineStr">
-        <is>
-          <t>0 / 23</t>
-        </is>
-      </c>
-      <c r="G17" s="67" t="inlineStr">
-        <is>
-          <t>ERROR 23</t>
-        </is>
-      </c>
-      <c r="H17" s="67" t="inlineStr">
-        <is>
-          <t>FAIL 23</t>
-        </is>
-      </c>
-      <c r="I17" s="68" t="inlineStr">
-        <is>
-          <t>PASS 23</t>
-        </is>
-      </c>
-      <c r="J17" s="67" t="inlineStr">
-        <is>
-          <t>FAIL 23</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="60" t="inlineStr">
-        <is>
-          <t>Over-specific cases (11): relaxed test valid on 148 / 148 pairs; LLM fix passes 148 / 148.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:I2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>